<commit_message>
Update reports 2026-09-14 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-14.xlsx
+++ b/gex_pivot_levels_2026-09-14.xlsx
@@ -622,743 +622,743 @@
       <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>7515.27</v>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>7550</v>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="A5" s="2" t="n">
+        <v>7505.27</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>7540</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>-$15.98M</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>+$16.34M</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-$4.34M</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>+$4.49M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
+        <v>7515.27</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>7550</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>-$18.43M</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>+$18.85M</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
         <v>7529.18</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B7" s="6" t="n">
         <v>755</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>-$5.17M</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>+$8.99M</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>7530.27</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>7565</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$4.75M</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>+$5.32M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-$5.40M</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$6.05M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
+    <row r="9">
+      <c r="A9" s="6" t="n">
         <v>7540.27</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B9" s="6" t="n">
         <v>7575</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>-$12.88M</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>+$15.03M</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>-$14.40M</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>+$16.81M</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>7550.27</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>7585</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$5.08M</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$7.02M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$5.62M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$7.76M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
+    <row r="11">
+      <c r="A11" s="6" t="n">
         <v>7555.27</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B11" s="6" t="n">
         <v>7590</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>-$9.36M</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>+$10.41M</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>-$10.28M</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>+$11.44M</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>7560.27</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>7595</v>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>-$4.15M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$7.08M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-$4.48M</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$7.65M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
+    <row r="13">
+      <c r="A13" s="6" t="n">
         <v>7565.27</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B13" s="6" t="n">
         <v>7600</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>-$20.47M</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>+$33.24M</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>-$21.78M</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>+$35.37M</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>7575.27</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>7610</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>-$8.30M</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>+$11.77M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
+        <v>7575.27</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>7610</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-$8.50M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$12.05M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>7579.27</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>760</v>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>-$1.33M</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>+$23.01M</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>7580.27</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B16" s="6" t="n">
         <v>7615</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>-$15.14M</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>+$17.75M</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>7590.27</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>7625</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>-$8.70M</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>+$14.80M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>-$8.27M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$14.07M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>7599.31</v>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B18" s="6" t="n">
         <v>762</v>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>+$11.04M</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>+$14.00M</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>7609.33</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>763</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>+$4.56M</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$6.82M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
+        <v>7609.33</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>+$4.56M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$6.82M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>7615.27</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>7650</v>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>+$878.10K</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>+$20.87M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>+$748.55K</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>+$17.79M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
         <v>7629.36</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B21" s="6" t="n">
         <v>765</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>+$27.57M</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>+$59.85M</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>7639.38</v>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>766</v>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>+$4.84M</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>+$6.34M</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>7640.27</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B23" s="2" t="n">
         <v>7675</v>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>+$3.98M</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>+$13.42M</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>+$3.14M</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>+$10.57M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>7649.4</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>767</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>+$16.14M</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>+$20.04M</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>7649.4</v>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>767</v>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>+$16.14M</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>+$20.04M</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>7665.27</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>7700</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>+$2.71M</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>+$5.87M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
+        <v>7665.27</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>+$2.17M</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>+$4.69M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>7669.44</v>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B26" s="2" t="n">
         <v>769</v>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>+$2.27M</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>+$3.93M</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="n">
+    <row r="27">
+      <c r="A27" s="6" t="n">
         <v>7679.46</v>
       </c>
-      <c r="B26" s="6" t="n">
+      <c r="B27" s="6" t="n">
         <v>770</v>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>+$10.77M</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>+$20.49M</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>7685.27</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>7720</v>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>+$3.95M</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>+$4.27M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G27"/>
@@ -4202,12 +4202,12 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>-$20.47M</t>
+          <t>-$21.78M</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>+$33.24M</t>
+          <t>+$35.37M</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -4370,38 +4370,42 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>7615.27</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>+$878.10K</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>+$20.87M</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="B8" s="6" t="n">
+        <v>7679.46</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>770</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>+$10.77M</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>+$20.49M</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -4410,10 +4414,10 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>7679.46</v>
+        <v>7649.4</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -4422,12 +4426,12 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>+$10.77M</t>
+          <t>+$16.14M</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>+$20.49M</t>
+          <t>+$20.04M</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -4448,24 +4452,24 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>7649.4</v>
+        <v>7515.27</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>767</v>
+        <v>7550</v>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>+$16.14M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>-$18.43M</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>+$20.04M</t>
+          <t>+$18.85M</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -4475,7 +4479,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4514,114 +4518,110 @@
       <c r="H11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="2" t="n">
+        <v>7615.27</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>+$748.55K</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>+$17.79M</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
         <v>7580.27</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>7615</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>-$15.14M</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>+$17.75M</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B14" s="2" t="n">
         <v>4276.08</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C14" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>-$831.87K</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>+$17.33M</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>4051.02</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>-$9.35M</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>+$16.50M</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -4630,10 +4630,10 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>7515.27</v>
+        <v>7540.27</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>7550</v>
+        <v>7575</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
@@ -4642,12 +4642,12 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>-$15.98M</t>
+          <t>-$14.40M</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>+$16.34M</t>
+          <t>+$16.81M</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -4662,76 +4662,76 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>4051.02</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>-$9.35M</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>+$16.50M</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>2927.46</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>291</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>-$7.81M</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>+$15.85M</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>2867.1</v>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>285</v>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>-$14.20M</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>+$15.32M</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4740,28 +4740,28 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>28814.52</v>
+        <v>2867.1</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>710</v>
+        <v>285</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>-$2.12M</t>
+          <t>-$14.20M</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>+$15.14M</t>
+          <t>+$15.32M</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -4778,28 +4778,28 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>7540.27</v>
+        <v>28814.52</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>7575</v>
+        <v>710</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>-$12.88M</t>
+          <t>-$2.12M</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>+$15.03M</t>
+          <t>+$15.14M</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -4832,12 +4832,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>-$8.70M</t>
+          <t>-$8.27M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$14.80M</t>
+          <t>+$14.07M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -4888,114 +4888,114 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>29225.34</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>720</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>+$5.93M</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>+$12.40M</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n">
-        <v>7640.27</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>7675</v>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="B23" s="2" t="n">
+        <v>7575.27</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>7610</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>+$3.98M</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>+$13.42M</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$8.50M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>+$12.05M</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>7555.27</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>7590</v>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>-$10.28M</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>+$11.44M</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>29225.34</v>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>720</v>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$5.93M</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>+$12.40M</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>7575.27</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>7610</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>-$8.30M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$11.77M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5038,42 +5038,38 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n">
-        <v>7555.27</v>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>7590</v>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="B26" s="2" t="n">
+        <v>7640.27</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>-$9.36M</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>+$10.41M</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>+$3.14M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$10.57M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -5120,10 +5116,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>7560.27</v>
+        <v>7550.27</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>7595</v>
+        <v>7585</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
@@ -5132,12 +5128,12 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>-$4.15M</t>
+          <t>-$5.62M</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+$7.08M</t>
+          <t>+$7.76M</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -5158,10 +5154,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7550.27</v>
+        <v>7560.27</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>7585</v>
+        <v>7595</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
@@ -5170,12 +5166,12 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>-$5.08M</t>
+          <t>-$4.48M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$7.02M</t>
+          <t>+$7.65M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -5272,32 +5268,36 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>7665.27</v>
+        <v>7530.27</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>7700</v>
+        <v>7565</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>+$2.71M</t>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>-$5.40M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$5.87M</t>
+          <t>+$6.05M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -5450,108 +5450,108 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>7530.27</v>
+        <v>7665.27</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7565</v>
+        <v>7700</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>-$4.75M</t>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>+$2.17M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$5.32M</t>
+          <t>+$4.69M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>7505.27</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>7540</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>-$4.34M</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>+$4.49M</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
+      <c r="B39" s="6" t="n">
         <v>28609.11</v>
       </c>
-      <c r="C38" s="6" t="n">
+      <c r="C39" s="6" t="n">
         <v>705</v>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>-$3.20M</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>+$4.48M</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>7685.27</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>7720</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>+$3.95M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$4.27M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">

</xml_diff>